<commit_message>
[P9] docs(usage): refresh Databricks spend to date and running-cost figures
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J4aRjEgFqM3dK34XuEwuYk
</commit_message>
<xml_diff>
--- a/docs/usage/token_usage_2026-09-24.xlsx
+++ b/docs/usage/token_usage_2026-09-24.xlsx
@@ -545,7 +545,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>The SQL warehouse ran all day at ~12 DBU/hour and never reached its 10-minute auto-stop, most likely because the App polls Delta every few seconds. At list price that is ~$218/day of the ~$231 total. Fixable: idle back-off in the App polling loop.</t>
+          <t>SQL warehouse: ~$241 on 2026-09-23, of which ~$218 was the idle-polling incident (the App kept the warehouse awake 02:00-22:00 UTC). Fixed 2026-09-24: no warehouse polling while idle, auto-stop 1 min. Measured afterwards: the warehouse still stops ~20 min after the last query (platform latency), so each burst of activity costs ~20 min of warehouse time. The App itself costs ~0.7 DBU (~$0.58) per hour while running, even when idle; stop it when not in use.</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3340,7 +3340,7 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="90" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3440,10 +3440,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>40.063</v>
+        <v>42.356</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>1.06</v>
       </c>
       <c r="F4" t="inlineStr"/>
     </row>
@@ -3466,6 +3466,9 @@
       <c r="D5" t="n">
         <v>0.231</v>
       </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
       <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
@@ -3581,10 +3584,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.21</v>
+        <v>0.358</v>
       </c>
       <c r="E10" t="n">
-        <v>0.17</v>
+        <v>0.3</v>
       </c>
       <c r="F10" t="inlineStr"/>
     </row>
@@ -3596,19 +3599,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NETWORKING</t>
+          <t>DEFAULT_STORAGE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>DSU</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.26</v>
+        <v>0.584</v>
       </c>
       <c r="E11" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="F11" t="inlineStr"/>
     </row>
@@ -3620,19 +3623,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PREDICTIVE_OPTIMIZATION</t>
+          <t>NETWORKING</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DBU</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.146</v>
+        <v>0.523</v>
       </c>
       <c r="E12" t="n">
-        <v>0.06</v>
+        <v>0.03</v>
       </c>
       <c r="F12" t="inlineStr"/>
     </row>
@@ -3644,7 +3647,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SQL</t>
+          <t>PREDICTIVE_OPTIMIZATION</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3653,27 +3656,193 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>9.635</v>
+        <v>0.341</v>
       </c>
       <c r="E13" t="n">
-        <v>9.15</v>
+        <v>0.13</v>
       </c>
       <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DBU</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>25.806</v>
+      </c>
+      <c r="E14" t="n">
+        <v>24.52</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BY PRODUCT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="E16" t="n">
+        <v>265.81</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BY PRODUCT</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>APPS</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>11.97</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BY PRODUCT</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PREDICTIVE_OPTIMIZATION</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BY PRODUCT</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>DEFAULT_STORAGE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BY PRODUCT</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>NETWORKING</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BY PRODUCT</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>AI_GATEWAY</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BY PRODUCT</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>GENIE</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BY PRODUCT</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>MODEL_SERVING</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="E14" t="n">
-        <v>264.5</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>billing posted through 2026-09-24 02:00:00+00:00 UTC; lags several hours</t>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>280.15</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>USD at Databricks list price; billing posted through 2026-09-24T08:00:00.000Z UTC and lags several hours. Your actual charge depends on your plan, discounts or trial credits.</t>
         </is>
       </c>
     </row>

</xml_diff>